<commit_message>
this is Complete Check Update
</commit_message>
<xml_diff>
--- a/Data/BeginingOfModernAge.xlsx
+++ b/Data/BeginingOfModernAge.xlsx
@@ -472,1451 +472,1451 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Who was the king of France at the time of the French Revolution?</t>
+          <t>Which century is known for the beginning of European colonialism in Asia?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Louis XVI</t>
+          <t>13th</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Napoleon</t>
+          <t>14th</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Louis XV</t>
+          <t>15th</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Henry IV</t>
+          <t>16th</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Louis XVI</t>
+          <t>16th</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Which thinker is known for the concept of "social contract"?</t>
+          <t>Which ideology became prominent in opposition to absolute monarchy?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Feudalism</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Locke</t>
+          <t>Republicanism</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Colonialism</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Montesquieu</t>
+          <t>Totalitarianism</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Republicanism</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Who authored "Two Treatises of Government"?</t>
+          <t>What ideology rose in response to the inequalities of Industrialization?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thomas Hobbes</t>
+          <t>Feudalism</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Montesquieu</t>
+          <t>Colonialism</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>John Locke</t>
+          <t>Socialism</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Adam Smith</t>
+          <t>Mercantilism</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>John Locke</t>
+          <t>Socialism</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Which invention by Gutenberg in the 15th century revolutionized communication in Europe?</t>
+          <t>What was a major effect of the Industrial Revolution on workers?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Steam engine</t>
+          <t>Higher status</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Printing press</t>
+          <t>Decline of cities</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Telescope</t>
+          <t>Factory jobs</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Typewriter</t>
+          <t>Slavery increase</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Printing press</t>
+          <t>Factory jobs</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The American Revolution was inspired by the ideas of the:</t>
+          <t>Which French philosopher criticized religious intolerance and injustice through satire?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Renaissance</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Scientific Revolution</t>
+          <t>Kant</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Enlightenment</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>Montesquieu</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Enlightenment</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>What was a direct impact of the Reformation in Europe?</t>
+          <t>Which revolutionary invention helped spread new ideas during the Renaissance?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>End of monarchy</t>
+          <t>Telegraph</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fall of Rome</t>
+          <t>Compass</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Decline of Church authority</t>
+          <t>Printing press</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Rise of feudalism</t>
+          <t>Microscope</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Decline of Church authority</t>
+          <t>Printing press</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Which battle in 1815 ended Napoleon's rule permanently?</t>
+          <t>Which explorer’s voyages marked the start of the Age of Discovery?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Austerlitz</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Trafalgar</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Waterloo</t>
+          <t>Magellan</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Cook</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Waterloo</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Which European monarch is considered the best example of absolutism?</t>
+          <t>Which revolution inspired movements in Latin America?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Napoleon</t>
+          <t>American Revolution</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Frederick the Great</t>
+          <t>Industrial Revolution</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Louis XIV</t>
+          <t>Scientific Revolution</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Henry VIII</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Louis XIV</t>
+          <t>American Revolution</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>The Renaissance began in which country during the 14th century?</t>
+          <t>Which movement challenged the authority of the Catholic Church in the 16th century?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Renaissance</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Industrial Revolution</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Enlightenment</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Which movement challenged the authority of the Catholic Church in the 16th century?</t>
+          <t>Which social group gained prominence after the Industrial Revolution?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Renaissance</t>
+          <t>Nobility</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>Peasants</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Industrial Revolution</t>
+          <t>Clergy</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Enlightenment</t>
+          <t>Bourgeoisie</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>Bourgeoisie</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>The Napoleonic Code was a reform of:</t>
+          <t>The Enlightenment emphasized the importance of:</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Taxation</t>
+          <t>Divine Right</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Judiciary</t>
+          <t>Tradition</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Land ownership</t>
+          <t>Reason</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Legal system</t>
+          <t>Monarchy</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Legal system</t>
+          <t>Reason</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Which class rose to prominence due to industrial capitalism?</t>
+          <t>What was a direct impact of the Reformation in Europe?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Clergy</t>
+          <t>End of monarchy</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nobility</t>
+          <t>Fall of Rome</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Middle class</t>
+          <t>Decline of Church authority</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Peasants</t>
+          <t>Rise of feudalism</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Middle class</t>
+          <t>Decline of Church authority</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Who developed the three laws of planetary motion?</t>
+          <t>Voltaire was a fierce critic of which institution?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>The army</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Monarchs</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kepler</t>
+          <t>The Church</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Brahe</t>
+          <t>Merchants</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Kepler</t>
+          <t>The Church</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The Encyclopédie, a major Enlightenment work, was edited by:</t>
+          <t>Who authored "Two Treatises of Government"?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Thomas Hobbes</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Montesquieu</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Diderot</t>
+          <t>John Locke</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Locke</t>
+          <t>Adam Smith</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Diderot</t>
+          <t>John Locke</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>What ideology rose in response to the inequalities of Industrialization?</t>
+          <t>Who was the leading astronomer who proved the heliocentric theory with a telescope?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Feudalism</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Colonialism</t>
+          <t>Copernicus</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Socialism</t>
+          <t>Kepler</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Mercantilism</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Socialism</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The Boston Tea Party was a protest against:</t>
+          <t>Which Enlightenment thinker promoted religious tolerance and freedom of speech?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Slavery</t>
+          <t>Locke</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Religious oppression</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>British taxes</t>
+          <t>Kant</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Land policies</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>British taxes</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The Industrial Revolution began in which country?</t>
+          <t>Which empire colonized large parts of the Americas in the 16th century?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Ottoman</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Spanish</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Dutch</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>German</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Spanish</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Which invention greatly increased textile production during the Industrial Revolution?</t>
+          <t>Which economic theory dominated Europe before the Industrial Revolution?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Spinning Jenny</t>
+          <t>Capitalism</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Steam Engine</t>
+          <t>Mercantilism</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Cotton Gin</t>
+          <t>Feudalism</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Power Loom</t>
+          <t>Socialism</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Spinning Jenny</t>
+          <t>Mercantilism</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The slogan “Liberty, Equality, Fraternity” is associated with which revolution?</t>
+          <t>What was the Estates-General in France?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>A religious group</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>American</t>
+          <t>Royal court</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>French</t>
+          <t>Representative assembly</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Russian</t>
+          <t>Army unit</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>French</t>
+          <t>Representative assembly</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Which of the following was a major colonial power in the 17th century?</t>
+          <t>Which revolution is also called the "Age of Reason"?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Scientific Revolution</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Industrial Revolution</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>French Revolution</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Enlightenment</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Enlightenment</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Which ideology became prominent in opposition to absolute monarchy?</t>
+          <t>Which Enlightenment philosopher influenced the U.S. Constitution?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Feudalism</t>
+          <t>Locke</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Republicanism</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Colonialism</t>
+          <t>Kant</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Totalitarianism</t>
+          <t>Hobbes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Republicanism</t>
+          <t>Locke</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Which French philosopher criticized religious intolerance and injustice through satire?</t>
+          <t>Which invention by Gutenberg in the 15th century revolutionized communication in Europe?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Steam engine</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kant</t>
+          <t>Printing press</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Telescope</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Montesquieu</t>
+          <t>Typewriter</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Printing press</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Which Enlightenment thinker believed in the idea of general will?</t>
+          <t>What was the Estates System in France based on?</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Locke</t>
+          <t>Race</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Occupation</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Wealth</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Montesquieu</t>
+          <t>Social class</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Social class</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>The Reign of Terror in France was led by which revolutionary leader?</t>
+          <t>The Renaissance began in which country during the 14th century?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Napoleon</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Robespierre</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Danton</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Lafayette</t>
+          <t>England</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Robespierre</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>The American Declaration of Independence was signed in:</t>
+          <t>Who wrote the 95 Theses that sparked the Protestant Reformation?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>Calvin</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>Luther</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1815</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1757</t>
+          <t>Hobbes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>Luther</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>What was the Estates-General in France?</t>
+          <t>The ‘Storming of the Bastille’ became a symbol of:</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>A religious group</t>
+          <t>Royal power</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Royal court</t>
+          <t>Church authority</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Representative assembly</t>
+          <t>Revolutionary uprising</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Army unit</t>
+          <t>Economic crisis</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Representative assembly</t>
+          <t>Revolutionary uprising</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>The Enlightenment thinker Immanuel Kant is best known for his work on:</t>
+          <t>The Napoleonic Code was a reform of:</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Political liberty</t>
+          <t>Taxation</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Scientific method</t>
+          <t>Judiciary</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Moral philosophy</t>
+          <t>Land ownership</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Religious reform</t>
+          <t>Legal system</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Moral philosophy</t>
+          <t>Legal system</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Which revolution inspired movements in Latin America?</t>
+          <t>Which scientific thinker was tried for heresy by the Church?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>American Revolution</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Industrial Revolution</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Scientific Revolution</t>
+          <t>Kepler</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>Descartes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>American Revolution</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Who is known for formulating the laws of motion and universal gravitation?</t>
+          <t>The Renaissance focused primarily on:</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>Religious reform</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Kepler</t>
+          <t>Scientific inquiry</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Human potential and achievements</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Descartes</t>
+          <t>Economic planning</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Human potential and achievements</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Who proposed the heliocentric theory that placed the Sun at the center of the universe?</t>
+          <t>Which nation led the Age of Exploration with early maritime expeditions?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ptolemy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Copernicus</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Kepler</t>
+          <t>England</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Copernicus</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>The Renaissance focused primarily on:</t>
+          <t>The slogan “Liberty, Equality, Fraternity” is associated with which revolution?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Religious reform</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Scientific inquiry</t>
+          <t>American</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Human potential and achievements</t>
+          <t>French</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Economic planning</t>
+          <t>Russian</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Human potential and achievements</t>
+          <t>French</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Which thinker influenced both American and French Revolutions with his ideas on liberty?</t>
+          <t>Which class rose to prominence due to industrial capitalism?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Clergy</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Nobility</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Kant</t>
+          <t>Middle class</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Hegel</t>
+          <t>Peasants</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Middle class</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Which event marked the beginning of the French Revolution?</t>
+          <t>Who proposed the heliocentric theory that placed the Sun at the center of the universe?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Storming of the Bastille</t>
+          <t>Ptolemy</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Execution of Louis XVI</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tennis Court Oath</t>
+          <t>Copernicus</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Reign of Terror</t>
+          <t>Kepler</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Storming of the Bastille</t>
+          <t>Copernicus</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Which English philosopher wrote "Leviathan" advocating a strong central authority?</t>
+          <t>The Industrial Revolution began in which country?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>John Locke</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Thomas Hobbes</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>England</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Thomas Hobbes</t>
+          <t>England</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Which Enlightenment thinker promoted religious tolerance and freedom of speech?</t>
+          <t>The term “laissez-faire” economics is associated with which economist?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Locke</t>
+          <t>Keynes</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Marx</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Kant</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Ricardo</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Which revolution is also called the "Age of Reason"?</t>
+          <t>The first country to industrialize was:</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Scientific Revolution</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Industrial Revolution</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>French Revolution</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Enlightenment</t>
+          <t>Britain</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Enlightenment</t>
+          <t>Britain</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Who is known as the 'Father of Humanism'?</t>
+          <t>What marked the shift from manual labor to machine-based production?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Dante</t>
+          <t>Renaissance</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Erasmus</t>
+          <t>Enlightenment</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Petrarch</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Industrial Revolution</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Petrarch</t>
+          <t>Industrial Revolution</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Napoleon Bonaparte rose to power after which major event?</t>
+          <t>Who was the king of France at the time of the French Revolution?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Industrial Revolution</t>
+          <t>Louis XVI</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>French Revolution</t>
+          <t>Napoleon</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>American War</t>
+          <t>Louis XV</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>Henry IV</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>French Revolution</t>
+          <t>Louis XVI</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The Treaty of Westphalia (1648) ended which war?</t>
+          <t>Which major global shift began around 1500 CE?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>French Revolution</t>
+          <t>Age of Empires</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Thirty Years’ War</t>
+          <t>Dark Ages</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>American Revolution</t>
+          <t>Age of Exploration</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Napoleonic Wars</t>
+          <t>Age of Enlightenment</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Thirty Years’ War</t>
+          <t>Age of Exploration</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Which event ended the absolute monarchy in England and led to parliamentary democracy?</t>
+          <t>Which Enlightenment thinker advocated for the separation of powers?</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Glorious Revolution</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Civil War</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Magna Carta</t>
+          <t>Montesquieu</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>Kant</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Glorious Revolution</t>
+          <t>Montesquieu</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Which Enlightenment thinker advocated for the separation of powers?</t>
+          <t>Which thinker is known for the concept of "social contract"?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1926,274 +1926,274 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
+          <t>Locke</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
           <t>Rousseau</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Montesquieu</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Kant</t>
-        </is>
-      </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Montesquieu</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Who was the monarch during England's Glorious Revolution?</t>
+          <t>The Reign of Terror in France was led by which revolutionary leader?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Elizabeth I</t>
+          <t>Napoleon</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>George I</t>
+          <t>Robespierre</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>James II</t>
+          <t>Danton</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Henry VIII</t>
+          <t>Lafayette</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>James II</t>
+          <t>Robespierre</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Which explorer first circumnavigated the globe?</t>
+          <t>The factory system replaced which system of production?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Craft system</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Magellan</t>
+          <t>Feudal system</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Drake</t>
+          <t>Cottage industry</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Cook</t>
+          <t>Agrarian system</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Magellan</t>
+          <t>Cottage industry</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>What was the Estates System in France based on?</t>
+          <t>Which treaty ended the American Revolutionary War?</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Race</t>
+          <t>Treaty of Paris 1763</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Occupation</t>
+          <t>Treaty of Versailles</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Wealth</t>
+          <t>Treaty of Paris 1783</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Social class</t>
+          <t>Treaty of Ghent</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Social class</t>
+          <t>Treaty of Paris 1783</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>The ‘Storming of the Bastille’ became a symbol of:</t>
+          <t>Who is known for formulating the laws of motion and universal gravitation?</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Royal power</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Church authority</t>
+          <t>Kepler</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Revolutionary uprising</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Economic crisis</t>
+          <t>Descartes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Revolutionary uprising</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>The term “laissez-faire” economics is associated with which economist?</t>
+          <t>Which of the following was a cause of the French Revolution?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Keynes</t>
+          <t>Scientific inventions</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Marx</t>
+          <t>Colonialism</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Economic crisis and inequality</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Ricardo</t>
+          <t>Religious conversion</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Economic crisis and inequality</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Which Enlightenment idea directly challenged the Divine Right of Kings?</t>
+          <t>The Encyclopédie, a major Enlightenment work, was edited by:</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Religious dogma</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Social contract</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Natural rights</t>
+          <t>Diderot</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Democracy</t>
+          <t>Locke</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Social contract</t>
+          <t>Diderot</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Which treaty ended the American Revolutionary War?</t>
+          <t>Which event ended the absolute monarchy in England and led to parliamentary democracy?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Treaty of Paris 1763</t>
+          <t>Glorious Revolution</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Treaty of Versailles</t>
+          <t>Civil War</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Treaty of Paris 1783</t>
+          <t>Magna Carta</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Treaty of Ghent</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Treaty of Paris 1783</t>
+          <t>Glorious Revolution</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -2236,237 +2236,237 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Which thinker is known as the "father of modern economics"?</t>
+          <t>Which of the following was a major colonial power in the 17th century?</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Karl Marx</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>John Maynard Keynes</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Adam Smith</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>David Ricardo</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Adam Smith</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Which century is known for the beginning of European colonialism in Asia?</t>
+          <t>The Industrial Revolution primarily contributed to:</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>13th</t>
+          <t>Decline of trade</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>14th</t>
+          <t>Growth of agriculture</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>15th</t>
+          <t>Urbanization</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>16th</t>
+          <t>Feudal system</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>16th</t>
+          <t>Urbanization</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>The Industrial Revolution primarily contributed to:</t>
+          <t>Which battle in 1815 ended Napoleon's rule permanently?</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Decline of trade</t>
+          <t>Austerlitz</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Growth of agriculture</t>
+          <t>Trafalgar</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Urbanization</t>
+          <t>Waterloo</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Feudal system</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Urbanization</t>
+          <t>Waterloo</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Which political ideology gained momentum after the French Revolution?</t>
+          <t>Napoleon Bonaparte rose to power after which major event?</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Feudalism</t>
+          <t>Industrial Revolution</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Absolutism</t>
+          <t>French Revolution</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Republicanism</t>
+          <t>American War</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Colonialism</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Republicanism</t>
+          <t>French Revolution</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Which nation led the Age of Exploration with early maritime expeditions?</t>
+          <t>Which event marked the beginning of the French Revolution?</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Storming of the Bastille</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Execution of Louis XVI</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Tennis Court Oath</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Reign of Terror</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Storming of the Bastille</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>The factory system replaced which system of production?</t>
+          <t>The Enlightenment thinker Immanuel Kant is best known for his work on:</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Craft system</t>
+          <t>Political liberty</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Feudal system</t>
+          <t>Scientific method</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Cottage industry</t>
+          <t>Moral philosophy</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Agrarian system</t>
+          <t>Religious reform</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Cottage industry</t>
+          <t>Moral philosophy</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Which Enlightenment philosopher influenced the U.S. Constitution?</t>
+          <t>Which thinker influenced both American and French Revolutions with his ideas on liberty?</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Locke</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2476,696 +2476,696 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Hobbes</t>
+          <t>Hegel</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Locke</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>74</v>
+        <v>3</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Which of the following was a cause of the French Revolution?</t>
+          <t>Who is known as the 'Father of Humanism'?</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Scientific inventions</t>
+          <t>Dante</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Colonialism</t>
+          <t>Erasmus</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Economic crisis and inequality</t>
+          <t>Petrarch</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Religious conversion</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Economic crisis and inequality</t>
+          <t>Petrarch</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Which major global shift began around 1500 CE?</t>
+          <t>Who developed the three laws of planetary motion?</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Age of Empires</t>
+          <t>Galileo</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Dark Ages</t>
+          <t>Newton</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Age of Exploration</t>
+          <t>Kepler</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Age of Enlightenment</t>
+          <t>Brahe</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Age of Exploration</t>
+          <t>Kepler</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Which economic theory dominated Europe before the Industrial Revolution?</t>
+          <t>The Treaty of Westphalia (1648) ended which war?</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Capitalism</t>
+          <t>French Revolution</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mercantilism</t>
+          <t>Thirty Years’ War</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Feudalism</t>
+          <t>American Revolution</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Socialism</t>
+          <t>Napoleonic Wars</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Mercantilism</t>
+          <t>Thirty Years’ War</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>The Enlightenment period is also known as the:</t>
+          <t>Which English philosopher wrote "Leviathan" advocating a strong central authority?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Dark Age</t>
+          <t>John Locke</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Age of Reason</t>
+          <t>Thomas Hobbes</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Age of Faith</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Age of War</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Age of Reason</t>
+          <t>Thomas Hobbes</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Who was the leading astronomer who proved the heliocentric theory with a telescope?</t>
+          <t>The Boston Tea Party was a protest against:</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Slavery</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Copernicus</t>
+          <t>Religious oppression</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Kepler</t>
+          <t>British taxes</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>Land policies</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>British taxes</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Who wrote the 95 Theses that sparked the Protestant Reformation?</t>
+          <t>Which Enlightenment thinker believed in the idea of general will?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Calvin</t>
+          <t>Locke</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Luther</t>
+          <t>Voltaire</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Voltaire</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Hobbes</t>
+          <t>Montesquieu</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Luther</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Which scientific thinker was tried for heresy by the Church?</t>
+          <t>Who invented the steam engine that powered the Industrial Revolution?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>James Watt</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Eli Whitney</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Kepler</t>
+          <t>Thomas Edison</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Descartes</t>
+          <t>Robert Fulton</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Galileo</t>
+          <t>James Watt</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Which social group gained prominence after the Industrial Revolution?</t>
+          <t>The American Revolution was inspired by the ideas of the:</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Nobility</t>
+          <t>Renaissance</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Peasants</t>
+          <t>Scientific Revolution</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Clergy</t>
+          <t>Enlightenment</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Bourgeoisie</t>
+          <t>Reformation</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Bourgeoisie</t>
+          <t>Enlightenment</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>The first factory in the world was set up in which industry?</t>
+          <t>Which explorer first circumnavigated the globe?</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Cotton textiles</t>
+          <t>Magellan</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Coal</t>
+          <t>Drake</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Cook</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Cotton textiles</t>
+          <t>Magellan</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>What was a major effect of the Industrial Revolution on workers?</t>
+          <t>Which political ideology gained momentum after the French Revolution?</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Higher status</t>
+          <t>Feudalism</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Decline of cities</t>
+          <t>Absolutism</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Factory jobs</t>
+          <t>Republicanism</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Slavery increase</t>
+          <t>Colonialism</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Factory jobs</t>
+          <t>Republicanism</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Which empire colonized large parts of the Americas in the 16th century?</t>
+          <t>Who was the monarch during England's Glorious Revolution?</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Ottoman</t>
+          <t>Elizabeth I</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>George I</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Dutch</t>
+          <t>James II</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Henry VIII</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>James II</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Which event symbolized the end of feudalism in France?</t>
+          <t>Which thinker is known as the "father of modern economics"?</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Reign of Terror</t>
+          <t>Karl Marx</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Storming of the Bastille</t>
+          <t>John Maynard Keynes</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Execution of Robespierre</t>
+          <t>Adam Smith</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Napoleonic Wars</t>
+          <t>David Ricardo</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Storming of the Bastille</t>
+          <t>Adam Smith</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>What marked the shift from manual labor to machine-based production?</t>
+          <t>The American Declaration of Independence was signed in:</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Renaissance</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Enlightenment</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Reformation</t>
+          <t>1815</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Industrial Revolution</t>
+          <t>1757</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Industrial Revolution</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Which explorer’s voyages marked the start of the Age of Discovery?</t>
+          <t>Which Enlightenment idea directly challenged the Divine Right of Kings?</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Religious dogma</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Social contract</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Magellan</t>
+          <t>Natural rights</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Cook</t>
+          <t>Democracy</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Social contract</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>The first country to industrialize was:</t>
+          <t>Which invention greatly increased textile production during the Industrial Revolution?</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spinning Jenny</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Steam Engine</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Cotton Gin</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Power Loom</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Spinning Jenny</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Which revolutionary invention helped spread new ideas during the Renaissance?</t>
+          <t>The Enlightenment period is also known as the:</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Telegraph</t>
+          <t>Dark Age</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Compass</t>
+          <t>Age of Reason</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Printing press</t>
+          <t>Age of Faith</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Microscope</t>
+          <t>Age of War</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Printing press</t>
+          <t>Age of Reason</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>6</v>
+        <v>66</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>The Enlightenment emphasized the importance of:</t>
+          <t>Which event symbolized the end of feudalism in France?</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Divine Right</t>
+          <t>Reign of Terror</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Tradition</t>
+          <t>Storming of the Bastille</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Execution of Robespierre</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Monarchy</t>
+          <t>Napoleonic Wars</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Storming of the Bastille</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Voltaire was a fierce critic of which institution?</t>
+          <t>The first factory in the world was set up in which industry?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The army</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Monarchs</t>
+          <t>Cotton textiles</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>The Church</t>
+          <t>Coal</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Merchants</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>The Church</t>
+          <t>Cotton textiles</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Who invented the steam engine that powered the Industrial Revolution?</t>
+          <t>Which European monarch is considered the best example of absolutism?</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>James Watt</t>
+          <t>Napoleon</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Eli Whitney</t>
+          <t>Frederick the Great</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Thomas Edison</t>
+          <t>Louis XIV</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Robert Fulton</t>
+          <t>Henry VIII</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>James Watt</t>
+          <t>Louis XIV</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>

</xml_diff>